<commit_message>
Refactor RFM Excel export script for clarity and add segment summary functionality
</commit_message>
<xml_diff>
--- a/output/rfm_analysis.xlsx
+++ b/output/rfm_analysis.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="RFM Analysis" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Segment Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F103"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -3065,4 +3066,110 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Customer Count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Average Order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C2" t="n">
+        <v>7638832</v>
+      </c>
+      <c r="D2" t="n">
+        <v>190970.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Loyal</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2938882</v>
+      </c>
+      <c r="D3" t="n">
+        <v>127777.4782608696</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1903380</v>
+      </c>
+      <c r="D4" t="n">
+        <v>79307.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>At Risk</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" t="n">
+        <v>279757</v>
+      </c>
+      <c r="D5" t="n">
+        <v>21519.76923076923</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>